<commit_message>
add AggNo, fire downgarde logic
</commit_message>
<xml_diff>
--- a/Grading template formulation (2).xlsx
+++ b/Grading template formulation (2).xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30502"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://farmerschoice-my.sharepoint.com/personal/emuga_farmerschoice_co_ke/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\fcl\cml-calibra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BD475DD-30C4-486F-8F83-D35BE054D207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99676120-B37B-4CDC-86AF-C2B38DBD511E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="2" xr2:uid="{A813A2DF-C5EE-4228-AF12-C0706CB8B14B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" firstSheet="2" activeTab="4" xr2:uid="{A813A2DF-C5EE-4228-AF12-C0706CB8B14B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="BEST CASE" sheetId="3" r:id="rId3"/>
     <sheet name="WORST CASE" sheetId="4" r:id="rId4"/>
+    <sheet name="Lamb Grading" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="95">
   <si>
     <t>Fat cover</t>
   </si>
@@ -294,13 +295,46 @@
   </si>
   <si>
     <t>170kgs-199.9kgs</t>
+  </si>
+  <si>
+    <t>Class 1</t>
+  </si>
+  <si>
+    <t>Class 2</t>
+  </si>
+  <si>
+    <t>Class R</t>
+  </si>
+  <si>
+    <t>Any severely bruised lamb automatically grades as R without considering all other factors</t>
+  </si>
+  <si>
+    <t>Any deep yellow fat colour lamb automatically grades as R without cosnidering any other factors</t>
+  </si>
+  <si>
+    <t>Any poorly conformed carcass automatically grades as R without cosnidering any other factors</t>
+  </si>
+  <si>
+    <t>14kgs-30kgs</t>
+  </si>
+  <si>
+    <t>11kgs-13.9kgs</t>
+  </si>
+  <si>
+    <t>Any Carcass above 30 kgs automatically grades as class 2 without considering any other factors</t>
+  </si>
+  <si>
+    <t>Below 11kgs</t>
+  </si>
+  <si>
+    <t>Any Carcass below 11 kgs automatically grades as R without considering any other factors</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -421,7 +455,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -481,6 +515,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -817,12 +854,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B59D8E12-3AFC-48AC-93E5-15B610844C10}">
   <dimension ref="B2:K20"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.35">
       <c r="D2" s="19" t="s">
         <v>0</v>
       </c>
@@ -835,7 +872,7 @@
       <c r="J2" s="19"/>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="2:11">
+    <row r="3" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B3" s="18" t="s">
         <v>2</v>
       </c>
@@ -849,66 +886,66 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:11" s="1" customFormat="1">
+    <row r="4" spans="2:11" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B4" s="18"/>
       <c r="C4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="2:11">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B5" s="18"/>
       <c r="C5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="2:11">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B6" s="18"/>
       <c r="C6" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:11">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B7" s="18"/>
       <c r="C7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="2:11">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:11">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="2:11">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="2:11">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="2:11">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="2:2">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="2:2">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="2:2">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>12</v>
       </c>
@@ -930,10 +967,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B754F4B5-C111-4F74-BC0A-EB56C51DC9A5}">
   <dimension ref="B1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="2:3" ht="15" thickBot="1"/>
-    <row r="2" spans="2:3" ht="43.35" customHeight="1">
+    <row r="1" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:3" ht="43.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="20" t="s">
         <v>13</v>
       </c>
@@ -941,11 +978,11 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="2:3" ht="15" thickBot="1">
+    <row r="3" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="21"/>
       <c r="C3" s="23"/>
     </row>
-    <row r="4" spans="2:3" ht="63" customHeight="1">
+    <row r="4" spans="2:3" ht="63" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="20" t="s">
         <v>15</v>
       </c>
@@ -953,11 +990,11 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="15" thickBot="1">
+    <row r="5" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B5" s="21"/>
       <c r="C5" s="23"/>
     </row>
-    <row r="6" spans="2:3" ht="147" customHeight="1">
+    <row r="6" spans="2:3" ht="147" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="20" t="s">
         <v>17</v>
       </c>
@@ -965,11 +1002,11 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="15" thickBot="1">
+    <row r="7" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B7" s="21"/>
       <c r="C7" s="23"/>
     </row>
-    <row r="8" spans="2:3" ht="93.6" customHeight="1">
+    <row r="8" spans="2:3" ht="93.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="20" t="s">
         <v>19</v>
       </c>
@@ -977,11 +1014,11 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="2:3" ht="15" thickBot="1">
+    <row r="9" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B9" s="21"/>
       <c r="C9" s="23"/>
     </row>
-    <row r="10" spans="2:3" ht="43.35" customHeight="1">
+    <row r="10" spans="2:3" ht="43.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="20" t="s">
         <v>21</v>
       </c>
@@ -989,11 +1026,11 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="15" thickBot="1">
+    <row r="11" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B11" s="21"/>
       <c r="C11" s="23"/>
     </row>
-    <row r="12" spans="2:3" ht="110.45" customHeight="1">
+    <row r="12" spans="2:3" ht="110.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="20" t="s">
         <v>23</v>
       </c>
@@ -1001,24 +1038,24 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="2:3" ht="15" thickBot="1">
+    <row r="13" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B13" s="21"/>
       <c r="C13" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="B12:B13"/>
     <mergeCell ref="C12:C13"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -1030,16 +1067,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF2F5348-4A58-4B9F-B7FD-1C88BE8EF76A}">
   <dimension ref="A1:K49"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="19.140625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" customWidth="1"/>
-    <col min="4" max="4" width="8.85546875" style="2"/>
-    <col min="5" max="5" width="10.5703125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" customWidth="1"/>
+    <col min="2" max="2" width="19.1796875" style="8" customWidth="1"/>
+    <col min="3" max="3" width="18.1796875" customWidth="1"/>
+    <col min="4" max="4" width="8.81640625" style="2"/>
+    <col min="5" max="5" width="10.54296875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="8" customFormat="1">
+    <row r="1" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
       <c r="D1" s="12" t="s">
@@ -1064,7 +1101,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B2" s="15" t="s">
         <v>32</v>
       </c>
@@ -1077,7 +1114,7 @@
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="16" t="s">
         <v>33</v>
       </c>
@@ -1097,7 +1134,7 @@
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="16"/>
       <c r="B4" s="9"/>
       <c r="C4" s="5" t="s">
@@ -1113,7 +1150,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="16"/>
       <c r="B5" s="9"/>
       <c r="C5" s="5" t="s">
@@ -1139,7 +1176,7 @@
       </c>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="16"/>
       <c r="B6" s="9"/>
       <c r="C6" s="5" t="s">
@@ -1155,7 +1192,7 @@
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="16"/>
       <c r="B7" s="9"/>
       <c r="C7" s="5" t="s">
@@ -1173,7 +1210,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="16"/>
       <c r="B8" s="9"/>
       <c r="C8" s="6"/>
@@ -1185,7 +1222,7 @@
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="16"/>
       <c r="B9" s="7" t="s">
         <v>17</v>
@@ -1205,7 +1242,7 @@
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="16"/>
       <c r="B10" s="7"/>
       <c r="C10" s="3" t="s">
@@ -1225,7 +1262,7 @@
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="16"/>
       <c r="B11" s="7"/>
       <c r="C11" s="3" t="s">
@@ -1243,7 +1280,7 @@
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="16"/>
       <c r="B12" s="7"/>
       <c r="C12" s="3" t="s">
@@ -1263,7 +1300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="16"/>
       <c r="B13" s="7"/>
       <c r="C13" s="3" t="s">
@@ -1279,7 +1316,7 @@
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="16"/>
       <c r="B14" s="7"/>
       <c r="C14" s="3"/>
@@ -1291,7 +1328,7 @@
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="16"/>
       <c r="B15" s="7" t="s">
         <v>23</v>
@@ -1319,7 +1356,7 @@
       </c>
       <c r="J15" s="3"/>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="16"/>
       <c r="B16" s="7"/>
       <c r="C16" s="3" t="s">
@@ -1335,7 +1372,7 @@
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="16"/>
       <c r="B17" s="7"/>
       <c r="C17" s="3" t="s">
@@ -1353,7 +1390,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="16"/>
       <c r="B18" s="7"/>
       <c r="C18" s="3" t="s">
@@ -1371,7 +1408,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="16"/>
       <c r="B19" s="7"/>
       <c r="C19" s="3" t="s">
@@ -1387,7 +1424,7 @@
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="16"/>
       <c r="B20" s="7"/>
       <c r="C20" s="3"/>
@@ -1399,7 +1436,7 @@
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="16"/>
       <c r="B21" s="7" t="s">
         <v>49</v>
@@ -1425,7 +1462,7 @@
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="16"/>
       <c r="B22" s="7"/>
       <c r="C22" s="3" t="s">
@@ -1443,7 +1480,7 @@
       </c>
       <c r="J22" s="3"/>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="16"/>
       <c r="B23" s="7"/>
       <c r="C23" s="3" t="s">
@@ -1461,7 +1498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="16"/>
       <c r="B24" s="7"/>
       <c r="C24" s="3"/>
@@ -1473,7 +1510,7 @@
       <c r="I24" s="3"/>
       <c r="J24" s="3"/>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="16"/>
       <c r="B25" s="7" t="s">
         <v>53</v>
@@ -1503,7 +1540,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="16"/>
       <c r="B26" s="7"/>
       <c r="C26" s="3" t="s">
@@ -1519,7 +1556,7 @@
       <c r="I26" s="3"/>
       <c r="J26" s="3"/>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="16"/>
       <c r="B27" s="7"/>
       <c r="C27" s="3"/>
@@ -1531,7 +1568,7 @@
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="16"/>
       <c r="B28" s="7" t="s">
         <v>19</v>
@@ -1555,7 +1592,7 @@
       </c>
       <c r="J28" s="3"/>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="16"/>
       <c r="B29" s="7"/>
       <c r="C29" s="3" t="s">
@@ -1575,7 +1612,7 @@
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="16"/>
       <c r="B30" s="7"/>
       <c r="C30" s="3" t="s">
@@ -1593,7 +1630,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="16"/>
       <c r="B31" s="7"/>
       <c r="C31" s="3" t="s">
@@ -1625,7 +1662,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B32" s="7"/>
       <c r="C32" s="3"/>
       <c r="D32" s="4"/>
@@ -1636,7 +1673,7 @@
       <c r="I32" s="3"/>
       <c r="J32" s="3"/>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="16" t="s">
         <v>60</v>
       </c>
@@ -1663,7 +1700,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" s="16"/>
       <c r="B34" s="7"/>
       <c r="C34" s="3" t="s">
@@ -1684,7 +1721,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="35" spans="1:11">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" s="16"/>
       <c r="B35" s="7"/>
       <c r="C35" s="3" t="s">
@@ -1705,7 +1742,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="36" spans="1:11">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" s="16"/>
       <c r="B36" s="7"/>
       <c r="C36" s="3" t="s">
@@ -1726,7 +1763,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="37" spans="1:11">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" s="16"/>
       <c r="B37" s="7"/>
       <c r="C37" s="3" t="s">
@@ -1745,7 +1782,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="38" spans="1:11">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" s="16"/>
       <c r="B38" s="7"/>
       <c r="C38" s="3" t="s">
@@ -1774,7 +1811,7 @@
       </c>
       <c r="J38" s="3"/>
     </row>
-    <row r="39" spans="1:11">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" s="11"/>
       <c r="D39" s="14"/>
       <c r="E39" s="14"/>
@@ -1783,13 +1820,13 @@
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
     </row>
-    <row r="40" spans="1:11">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="D40" s="17" t="s">
         <v>72</v>
       </c>
       <c r="E40" s="17"/>
     </row>
-    <row r="41" spans="1:11">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="D41" s="2" t="s">
         <v>73</v>
       </c>
@@ -1800,7 +1837,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="42" spans="1:11">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="C42" t="s">
         <v>76</v>
       </c>
@@ -1814,7 +1851,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="43" spans="1:11">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="C43" t="s">
         <v>78</v>
       </c>
@@ -1828,7 +1865,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="44" spans="1:11">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="C44" t="s">
         <v>28</v>
       </c>
@@ -1842,7 +1879,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="45" spans="1:11">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="C45" t="s">
         <v>79</v>
       </c>
@@ -1856,7 +1893,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="46" spans="1:11">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="C46" t="s">
         <v>80</v>
       </c>
@@ -1870,7 +1907,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="49" spans="3:3">
+    <row r="49" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C49" t="s">
         <v>81</v>
       </c>
@@ -1893,14 +1930,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1AC6274-A7CC-44A1-B333-6D602CE93056}">
   <dimension ref="A1:K38"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="19.140625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" customWidth="1"/>
-    <col min="4" max="5" width="8.85546875" style="2"/>
+    <col min="2" max="2" width="19.1796875" style="8" customWidth="1"/>
+    <col min="3" max="3" width="18.1796875" customWidth="1"/>
+    <col min="4" max="5" width="8.81640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="8" customFormat="1">
+    <row r="1" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
       <c r="D1" s="12" t="s">
@@ -1925,7 +1962,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B2" s="15" t="s">
         <v>32</v>
       </c>
@@ -1938,7 +1975,7 @@
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="16" t="s">
         <v>33</v>
       </c>
@@ -1958,7 +1995,7 @@
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="16"/>
       <c r="B4" s="9"/>
       <c r="C4" s="5" t="s">
@@ -1974,7 +2011,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="16"/>
       <c r="B5" s="9"/>
       <c r="C5" s="5" t="s">
@@ -1990,7 +2027,7 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="16"/>
       <c r="B6" s="9"/>
       <c r="C6" s="5" t="s">
@@ -2008,7 +2045,7 @@
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="16"/>
       <c r="B7" s="9"/>
       <c r="C7" s="5" t="s">
@@ -2034,7 +2071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="16"/>
       <c r="B8" s="9"/>
       <c r="C8" s="6"/>
@@ -2046,7 +2083,7 @@
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="16"/>
       <c r="B9" s="7" t="s">
         <v>17</v>
@@ -2066,7 +2103,7 @@
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="16"/>
       <c r="B10" s="7"/>
       <c r="C10" s="3" t="s">
@@ -2084,7 +2121,7 @@
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="16"/>
       <c r="B11" s="7"/>
       <c r="C11" s="3" t="s">
@@ -2104,7 +2141,7 @@
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="16"/>
       <c r="B12" s="7"/>
       <c r="C12" s="3" t="s">
@@ -2124,7 +2161,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="16"/>
       <c r="B13" s="7"/>
       <c r="C13" s="3" t="s">
@@ -2140,7 +2177,7 @@
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="16"/>
       <c r="B14" s="7"/>
       <c r="C14" s="3"/>
@@ -2152,7 +2189,7 @@
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="16"/>
       <c r="B15" s="7" t="s">
         <v>23</v>
@@ -2174,7 +2211,7 @@
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="16"/>
       <c r="B16" s="7"/>
       <c r="C16" s="3" t="s">
@@ -2196,7 +2233,7 @@
       </c>
       <c r="J16" s="3"/>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="16"/>
       <c r="B17" s="7"/>
       <c r="C17" s="3" t="s">
@@ -2214,7 +2251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="16"/>
       <c r="B18" s="7"/>
       <c r="C18" s="3" t="s">
@@ -2232,7 +2269,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="16"/>
       <c r="B19" s="7"/>
       <c r="C19" s="3" t="s">
@@ -2248,7 +2285,7 @@
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="16"/>
       <c r="B20" s="7"/>
       <c r="C20" s="3"/>
@@ -2260,7 +2297,7 @@
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="16"/>
       <c r="B21" s="7" t="s">
         <v>49</v>
@@ -2280,7 +2317,7 @@
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="16"/>
       <c r="B22" s="7"/>
       <c r="C22" s="3" t="s">
@@ -2302,7 +2339,7 @@
       <c r="I22" s="3"/>
       <c r="J22" s="3"/>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="16"/>
       <c r="B23" s="7"/>
       <c r="C23" s="3" t="s">
@@ -2322,7 +2359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="16"/>
       <c r="B24" s="7"/>
       <c r="C24" s="3"/>
@@ -2334,7 +2371,7 @@
       <c r="I24" s="3"/>
       <c r="J24" s="3"/>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="16"/>
       <c r="B25" s="7" t="s">
         <v>53</v>
@@ -2356,7 +2393,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="16"/>
       <c r="B26" s="7"/>
       <c r="C26" s="3" t="s">
@@ -2380,7 +2417,7 @@
       </c>
       <c r="J26" s="3"/>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="16"/>
       <c r="B27" s="7"/>
       <c r="C27" s="3"/>
@@ -2392,7 +2429,7 @@
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="16"/>
       <c r="B28" s="7" t="s">
         <v>19</v>
@@ -2414,7 +2451,7 @@
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="16"/>
       <c r="B29" s="7"/>
       <c r="C29" s="3" t="s">
@@ -2436,7 +2473,7 @@
       </c>
       <c r="J29" s="3"/>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="16"/>
       <c r="B30" s="7"/>
       <c r="C30" s="3" t="s">
@@ -2454,7 +2491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="16"/>
       <c r="B31" s="7"/>
       <c r="C31" s="3" t="s">
@@ -2486,7 +2523,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B32" s="7"/>
       <c r="C32" s="3"/>
       <c r="D32" s="4"/>
@@ -2497,7 +2534,7 @@
       <c r="I32" s="3"/>
       <c r="J32" s="3"/>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="16" t="s">
         <v>60</v>
       </c>
@@ -2524,7 +2561,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" s="16"/>
       <c r="B34" s="7"/>
       <c r="C34" s="3" t="s">
@@ -2545,7 +2582,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="35" spans="1:11">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" s="16"/>
       <c r="B35" s="7"/>
       <c r="C35" s="3" t="s">
@@ -2566,7 +2603,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="36" spans="1:11">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" s="16"/>
       <c r="B36" s="7"/>
       <c r="C36" s="3" t="s">
@@ -2587,7 +2624,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="37" spans="1:11">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" s="16"/>
       <c r="B37" s="7"/>
       <c r="C37" s="3" t="s">
@@ -2606,7 +2643,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="38" spans="1:11">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" s="16"/>
       <c r="B38" s="7"/>
       <c r="C38" s="3" t="s">
@@ -2646,4 +2683,540 @@
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 Farmer's Choice - Public</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7472425C-B228-4D27-9FBB-5869CF720733}">
+  <dimension ref="A1:J31"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A1" s="7"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="15"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" s="9"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="4">
+        <v>3</v>
+      </c>
+      <c r="D4" s="4">
+        <v>3</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" s="7"/>
+      <c r="B5" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="4">
+        <v>2</v>
+      </c>
+      <c r="D5" s="4"/>
+      <c r="E5" s="3">
+        <v>2</v>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" s="7"/>
+      <c r="B6" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3">
+        <v>1</v>
+      </c>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" s="7"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="4">
+        <v>3</v>
+      </c>
+      <c r="D8" s="4">
+        <v>3</v>
+      </c>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" s="7"/>
+      <c r="B9" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="4">
+        <v>2</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="3">
+        <v>2</v>
+      </c>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" s="7"/>
+      <c r="B10" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="4">
+        <v>1</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3">
+        <v>1</v>
+      </c>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" s="7"/>
+      <c r="B11" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" s="4">
+        <v>1</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3">
+        <v>1</v>
+      </c>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" s="7"/>
+      <c r="B12" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="4">
+        <v>0</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3">
+        <v>0</v>
+      </c>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" s="7"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="4">
+        <v>3</v>
+      </c>
+      <c r="D14" s="4">
+        <v>3</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" s="7"/>
+      <c r="B15" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="4">
+        <v>2</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="3">
+        <v>2</v>
+      </c>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" s="7"/>
+      <c r="B16" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="4">
+        <v>1</v>
+      </c>
+      <c r="D16" s="4"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3">
+        <v>1</v>
+      </c>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" s="7"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" s="4">
+        <v>2</v>
+      </c>
+      <c r="D18" s="4">
+        <v>2</v>
+      </c>
+      <c r="E18" s="3">
+        <v>2</v>
+      </c>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19" s="7"/>
+      <c r="B19" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="4">
+        <v>1</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A20" s="7"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A21" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" s="4">
+        <v>3</v>
+      </c>
+      <c r="D21" s="4">
+        <v>3</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A22" s="7"/>
+      <c r="B22" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C22" s="4">
+        <v>2</v>
+      </c>
+      <c r="D22" s="4"/>
+      <c r="E22" s="3">
+        <v>2</v>
+      </c>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A23" s="7"/>
+      <c r="B23" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C23" s="4">
+        <v>1</v>
+      </c>
+      <c r="D23" s="4"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3">
+        <v>1</v>
+      </c>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A24" s="7"/>
+      <c r="B24" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4">
+        <f t="shared" ref="D24:F24" si="0">SUM(D4:D23)</f>
+        <v>14</v>
+      </c>
+      <c r="E24" s="4">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="F24" s="4">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" s="7"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C26" s="4">
+        <v>5</v>
+      </c>
+      <c r="D26" s="4">
+        <v>5</v>
+      </c>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A27" s="7"/>
+      <c r="B27" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C27" s="4">
+        <v>4</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="3">
+        <v>4</v>
+      </c>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A28" s="7"/>
+      <c r="B28" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C28" s="4">
+        <v>3</v>
+      </c>
+      <c r="D28" s="4"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3">
+        <v>3</v>
+      </c>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A29" s="7"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A30" s="7"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A31" s="7"/>
+      <c r="B31" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4">
+        <f>D24+SUM(D26:D30)</f>
+        <v>19</v>
+      </c>
+      <c r="E31" s="4">
+        <f>E24+SUM(E26:E30)</f>
+        <v>14</v>
+      </c>
+      <c r="F31" s="4">
+        <f>F24+SUM(F26:F30)</f>
+        <v>8</v>
+      </c>
+      <c r="G31" s="4">
+        <f>G24+SUM(G26:G30)</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="4">
+        <f>H24+SUM(H26:H30)</f>
+        <v>0</v>
+      </c>
+      <c r="I31" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:B2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>